<commit_message>
Refresh phc_discharges enriched dictionary for facilityname (v1.2.2)
Documentation-only companion to v1.2.1: the *_enriched.xlsx reference file
(display_label / skip_condition / public_* columns; not read by the
cleaning pipeline at runtime) hadn't been regenerated to include the
facilityname field added in v1.2.1. Re-ran both enrichment passes
(00c_enrich_dictionary_from_scripts.r, 00e_enrich_from_public_dictionary.r)
in the correct documented order and verified content-diffed every other
dictionary against a pre-run backup -- only this one file changed.
</commit_message>
<xml_diff>
--- a/cleaning_pipeline_R/dictionaries/dictionary_mwi_phc_discharges_enriched.xlsx
+++ b/cleaning_pipeline_R/dictionaries/dictionary_mwi_phc_discharges_enriched.xlsx
@@ -15335,54 +15335,53 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>birthweight_g</t>
+          <t>facilityname</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>facilityname.value</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>facilityname.label</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>Birth weight (g) -- canonical (derived)</t>
+          <t>Name of Facility</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>derived</t>
+          <t>dropdown</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>numeric</t>
+          <t>categorical</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>Derived (computed by cleaning pipeline Module 15)</t>
+          <t>Legacy (absent from current data-keys-metadata.json)</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>birthweight_g</t>
+          <t>facilityname</t>
         </is>
       </c>
       <c r="K141" t="b">
         <v>1</v>
       </c>
-      <c r="L141" t="inlineStr">
-        <is>
-          <t>grams</t>
-        </is>
-      </c>
       <c r="M141" t="b">
         <v>0</v>
       </c>
-      <c r="P141" t="n">
-        <v>300</v>
-      </c>
-      <c r="Q141" t="n">
-        <v>7000</v>
-      </c>
       <c r="R141" t="inlineStr">
         <is>
-          <t>Derived canonical birth weight (grams). Cleaning pipeline Module 15 computes coalesce(birthweight, bwt, bwtdis) -- three names for the same concept across Neotree form/script versions (bwtdis is birth weight despite its name; sources are identical where they overlap). Emitted in every dataset (NA where no source column is present). Originals retained. Use this column for low-birth-weight analysis. Not a raw field; no .value column.</t>
+          <t>Raw script field key is 'Facility'; absent from data-keys-metadata.json for phc_discharges despite being present in raw data (confirmed via neotree_scripts/mwi-scripts/NeoDischarge (PHC) - metadata.json). Registered as 'facilityname' (not 'facility') because the raw column collides with the reserved system 'facility' key column after suffix stripping; see cfg$reserved_column_renames in 00_setup.r, which renames Facility.value/.label to facilityname.value/.label in Module 01 before Module 07's duplicate-column logic can discard it in favour of the always-populated system column. Injected via LEGACY_VARIABLES 2026-08-24. ValueMaps (KRH-&gt;Kabudula Community Hospital, LH-&gt;Lumbadzi Health Center) added via VALUEMAP_PATCHES.</t>
         </is>
       </c>
       <c r="W141"/>
@@ -15427,12 +15426,12 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>discharge_weight_g</t>
+          <t>birthweight_g</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>Discharge / last-recorded weight (g) -- canonical (derived)</t>
+          <t>Birth weight (g) -- canonical (derived)</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
@@ -15452,7 +15451,7 @@
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>discharge_weight_g</t>
+          <t>birthweight_g</t>
         </is>
       </c>
       <c r="K142" t="b">
@@ -15474,7 +15473,7 @@
       </c>
       <c r="R142" t="inlineStr">
         <is>
-          <t>Derived canonical discharge / last-recorded weight (grams) = dischweight (date in datedischweight). Distinct concept from birth weight; never folded into it. Cleaning pipeline Module 15. Not a raw field; no .value column.</t>
+          <t>Derived canonical birth weight (grams). Cleaning pipeline Module 15 computes coalesce(birthweight, bwt, bwtdis) -- three names for the same concept across Neotree form/script versions (bwtdis is birth weight despite its name; sources are identical where they overlap). Emitted in every dataset (NA where no source column is present). Originals retained. Use this column for low-birth-weight analysis. Not a raw field; no .value column.</t>
         </is>
       </c>
       <c r="W142"/>
@@ -15519,12 +15518,12 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>mat_age_years_combined</t>
+          <t>discharge_weight_g</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>Maternal age (years) -- canonical (derived)</t>
+          <t>Discharge / last-recorded weight (g) -- canonical (derived)</t>
         </is>
       </c>
       <c r="G143" t="inlineStr">
@@ -15544,24 +15543,29 @@
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>mat_age_years_combined</t>
+          <t>discharge_weight_g</t>
         </is>
       </c>
       <c r="K143" t="b">
         <v>1</v>
       </c>
+      <c r="L143" t="inlineStr">
+        <is>
+          <t>grams</t>
+        </is>
+      </c>
       <c r="M143" t="b">
         <v>0</v>
       </c>
       <c r="P143" t="n">
-        <v>9</v>
+        <v>300</v>
       </c>
       <c r="Q143" t="n">
-        <v>60</v>
+        <v>7000</v>
       </c>
       <c r="R143" t="inlineStr">
         <is>
-          <t>Derived canonical maternal age in years. Cleaning pipeline Module 15 computes coalesce(matageyrs, mat_age_date_years): the manually entered whole-year field wins, falling back to the value derived from matagedate (auto-calculated from DOB, stored in HOURS, converted to years and range-filtered in Module 11). Both inputs are already range-clean (9-60), so this is a lossless coalesce plus a provenance label. Emitted only where at least one source column is present. Rows where both sources are present and disagree by more than 1 year are counted and logged, never overwritten -- see the per-run report 15b_maternal_age_summary.txt. Provenance is in mat_age_source. Originals retained. Not a raw field; no .value column.</t>
+          <t>Derived canonical discharge / last-recorded weight (grams) = dischweight (date in datedischweight). Distinct concept from birth weight; never folded into it. Cleaning pipeline Module 15. Not a raw field; no .value column.</t>
         </is>
       </c>
       <c r="W143"/>
@@ -15606,12 +15610,12 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>mat_age_source</t>
+          <t>mat_age_years_combined</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>Maternal age -- source of the derived value (provenance)</t>
+          <t>Maternal age (years) -- canonical (derived)</t>
         </is>
       </c>
       <c r="G144" t="inlineStr">
@@ -15621,7 +15625,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>categorical</t>
+          <t>numeric</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -15631,7 +15635,7 @@
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>mat_age_source</t>
+          <t>mat_age_years_combined</t>
         </is>
       </c>
       <c r="K144" t="b">
@@ -15640,9 +15644,15 @@
       <c r="M144" t="b">
         <v>0</v>
       </c>
+      <c r="P144" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q144" t="n">
+        <v>60</v>
+      </c>
       <c r="R144" t="inlineStr">
         <is>
-          <t>Provenance label for mat_age_years_combined, emitted alongside it by Module 15. One of: 'matageyrs' (manually entered whole years, the priority source), 'matagedate_derived' (converted from the auto-calculated DOB field in Module 11), or 'none' (neither source populated on that row). Use it to restrict an analysis to manually entered ages, or to quantify reliance on the derived fallback. Not a raw field; no .value column.</t>
+          <t>Derived canonical maternal age in years. Cleaning pipeline Module 15 computes coalesce(matageyrs, mat_age_date_years): the manually entered whole-year field wins, falling back to the value derived from matagedate (auto-calculated from DOB, stored in HOURS, converted to years and range-filtered in Module 11). Both inputs are already range-clean (9-60), so this is a lossless coalesce plus a provenance label. Emitted only where at least one source column is present. Rows where both sources are present and disagree by more than 1 year are counted and logged, never overwritten -- see the per-run report 15b_maternal_age_summary.txt. Provenance is in mat_age_source. Originals retained. Not a raw field; no .value column.</t>
         </is>
       </c>
       <c r="W144"/>
@@ -15671,6 +15681,87 @@
         <v>141</v>
       </c>
       <c r="AH144" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Malawi</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>MWI_phc_discharges</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>mat_age_source</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>Maternal age -- source of the derived value (provenance)</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>derived</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>Derived (computed by cleaning pipeline Module 15)</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>mat_age_source</t>
+        </is>
+      </c>
+      <c r="K145" t="b">
+        <v>1</v>
+      </c>
+      <c r="M145" t="b">
+        <v>0</v>
+      </c>
+      <c r="R145" t="inlineStr">
+        <is>
+          <t>Provenance label for mat_age_years_combined, emitted alongside it by Module 15. One of: 'matageyrs' (manually entered whole years, the priority source), 'matagedate_derived' (converted from the auto-calculated DOB field in Module 11), or 'none' (neither source populated on that row). Use it to restrict an analysis to manually entered ages, or to quantify reliance on the derived fallback. Not a raw field; no .value column.</t>
+        </is>
+      </c>
+      <c r="W145"/>
+      <c r="X145"/>
+      <c r="Y145"/>
+      <c r="Z145"/>
+      <c r="AA145" t="s">
+        <v>141</v>
+      </c>
+      <c r="AB145" t="s">
+        <v>141</v>
+      </c>
+      <c r="AC145" t="s">
+        <v>141</v>
+      </c>
+      <c r="AD145" t="s">
+        <v>141</v>
+      </c>
+      <c r="AE145" t="s">
+        <v>141</v>
+      </c>
+      <c r="AF145" t="s">
+        <v>141</v>
+      </c>
+      <c r="AG145" t="s">
+        <v>141</v>
+      </c>
+      <c r="AH145" t="b">
         <v>0</v>
       </c>
     </row>
@@ -45930,50 +46021,50 @@
     <row r="1009">
       <c r="A1009" t="inlineStr">
         <is>
-          <t>inorout</t>
+          <t>facilityname</t>
         </is>
       </c>
       <c r="B1009" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>KRH</t>
         </is>
       </c>
       <c r="C1009" t="inlineStr">
         <is>
-          <t>Inborn (legacy Yes)</t>
+          <t>Kabudula Community Hospital</t>
         </is>
       </c>
       <c r="D1009" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F1009" t="inlineStr">
         <is>
-          <t>In</t>
+          <t>KRH</t>
         </is>
       </c>
     </row>
     <row r="1010">
       <c r="A1010" t="inlineStr">
         <is>
-          <t>inorout</t>
+          <t>facilityname</t>
         </is>
       </c>
       <c r="B1010" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>LH</t>
         </is>
       </c>
       <c r="C1010" t="inlineStr">
         <is>
-          <t>Inborn (legacy true)</t>
+          <t>Lumbadzi Health Center</t>
         </is>
       </c>
       <c r="D1010" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F1010" t="inlineStr">
         <is>
-          <t>In</t>
+          <t>LH</t>
         </is>
       </c>
     </row>
@@ -45985,20 +46076,20 @@
       </c>
       <c r="B1011" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C1011" t="inlineStr">
         <is>
-          <t>Outborn (legacy No)</t>
+          <t>Inborn (legacy Yes)</t>
         </is>
       </c>
       <c r="D1011" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F1011" t="inlineStr">
         <is>
-          <t>Out</t>
+          <t>In</t>
         </is>
       </c>
     </row>
@@ -46010,18 +46101,68 @@
       </c>
       <c r="B1012" t="inlineStr">
         <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="C1012" t="inlineStr">
+        <is>
+          <t>Inborn (legacy true)</t>
+        </is>
+      </c>
+      <c r="D1012" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1012" t="inlineStr">
+        <is>
+          <t>In</t>
+        </is>
+      </c>
+    </row>
+    <row r="1013">
+      <c r="A1013" t="inlineStr">
+        <is>
+          <t>inorout</t>
+        </is>
+      </c>
+      <c r="B1013" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C1013" t="inlineStr">
+        <is>
+          <t>Outborn (legacy No)</t>
+        </is>
+      </c>
+      <c r="D1013" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1013" t="inlineStr">
+        <is>
+          <t>Out</t>
+        </is>
+      </c>
+    </row>
+    <row r="1014">
+      <c r="A1014" t="inlineStr">
+        <is>
+          <t>inorout</t>
+        </is>
+      </c>
+      <c r="B1014" t="inlineStr">
+        <is>
           <t>false</t>
         </is>
       </c>
-      <c r="C1012" t="inlineStr">
+      <c r="C1014" t="inlineStr">
         <is>
           <t>Outborn (legacy false)</t>
         </is>
       </c>
-      <c r="D1012" t="n">
+      <c r="D1014" t="n">
         <v>6</v>
       </c>
-      <c r="F1012" t="inlineStr">
+      <c r="F1014" t="inlineStr">
         <is>
           <t>Out</t>
         </is>

</xml_diff>